<commit_message>
update code to compatible with pytest
</commit_message>
<xml_diff>
--- a/data/test_cases/account_test_cases.xlsx
+++ b/data/test_cases/account_test_cases.xlsx
@@ -14,12 +14,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="55">
+  <si>
+    <t>case_no</t>
+  </si>
   <si>
     <t>status</t>
   </si>
   <si>
-    <t>case_no</t>
+    <t>priority</t>
+  </si>
+  <si>
+    <t>case_type</t>
   </si>
   <si>
     <t>author</t>
@@ -52,10 +58,16 @@
     <t>note</t>
   </si>
   <si>
+    <t>Account01</t>
+  </si>
+  <si>
     <t>Done</t>
   </si>
   <si>
-    <t>Account01</t>
+    <t>critical</t>
+  </si>
+  <si>
+    <t>positive</t>
   </si>
   <si>
     <t>Nhat</t>
@@ -91,19 +103,13 @@
     <t>/api/accounts/{admin_account_id}</t>
   </si>
   <si>
-    <t>{"_id":"{admin_account_id}","status_code":300}</t>
-  </si>
-  <si>
-    <t>For test write data to report, correct status_code is 200.</t>
+    <t/>
   </si>
   <si>
     <t>Account03</t>
   </si>
   <si>
-    <t>CreateNewRole</t>
-  </si>
-  <si>
-    <t>Create new account with role student.</t>
+    <t>Create new account with role admin.</t>
   </si>
   <si>
     <t>POST</t>
@@ -118,12 +124,12 @@
     <t>{"status_code":200}</t>
   </si>
   <si>
-    <t>Skip</t>
-  </si>
-  <si>
     <t>Account04</t>
   </si>
   <si>
+    <t>major</t>
+  </si>
+  <si>
     <t>Edit current student account.</t>
   </si>
   <si>
@@ -133,13 +139,46 @@
     <t>/api/accounts/{account_01_id}</t>
   </si>
   <si>
-    <t>{"role_name": "{student_role_name}", "full_name": "API predata - student account 01 - edited", "date_of_birth": "{datetime(%Y-%m-%d,0)}", "gender": "nam", "address": "API predata - student account 01 - address", "email": "api_predata_admin_account_01@gmail.com", "phone_number": "1234567890", "password": "123456789", "confirmPassword": "123456789", "is_deleted": false, "avatar": ""}</t>
+    <t>{"_id":"{account_01_id}","role_name": "{student_role_name}", "full_name": "API predata - student account 01 - edited", "date_of_birth": "{datetime(%Y-%m-%d,0)}", "gender": "nam", "address": "API predata - student account 01 - address", "email": "api_predata_admin_account_01@gmail.com", "phone_number": "1234567890", "password": "123456789", "confirmPassword": "123456789", "is_deleted": false, "avatar": ""}</t>
   </si>
   <si>
     <t>{"_id":"{account_01_id}","status_code":200}</t>
   </si>
   <si>
-    <t>Due to system config, can not edit account.</t>
+    <t>Due to system config, can not edit account. So this case always fail.</t>
+  </si>
+  <si>
+    <t>Account05</t>
+  </si>
+  <si>
+    <t>student</t>
+  </si>
+  <si>
+    <t>Get all accounts with student role.</t>
+  </si>
+  <si>
+    <t>Account06</t>
+  </si>
+  <si>
+    <t>teacher</t>
+  </si>
+  <si>
+    <t>Get all accounts with teacher role.</t>
+  </si>
+  <si>
+    <t>Account07</t>
+  </si>
+  <si>
+    <t>negative</t>
+  </si>
+  <si>
+    <t>Create new account with role teacher.</t>
+  </si>
+  <si>
+    <t>{"role_name": "{student_role_name}", "full_name": "API csv - student account 02", "date_of_birth": "2022-01-25", "gender": "nam", "address": "API csv - student account 02 - address", "email": "api_csv_student_account_02@gmail.com", "phone_number": "1234567890", "password": "123456789", "confirmPassword": "123456789"}</t>
+  </si>
+  <si>
+    <t>{"status_code":401}</t>
   </si>
 </sst>
 </file>
@@ -176,9 +215,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -486,21 +528,23 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="2" width="6.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="2" width="12.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="2" width="7.433571428571429" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="2" width="6.433571428571429" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="2" width="13.576428571428572" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="6" max="6" style="2" width="49.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="2" width="10.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="2" width="29.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="2" width="59.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="2" width="51.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="2" width="47.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="3" width="10.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="3" width="7.433571428571429" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="3" width="8.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="3" width="13.576428571428572" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="8" max="8" style="3" width="49.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="3" width="10.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="3" width="29.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="3" width="340.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="3" width="51.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="3" width="47.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -540,95 +584,111 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" s="1"/>
+        <v>21</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>22</v>
+      </c>
       <c r="J2" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
+      <c r="L2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
+      </c>
+      <c r="M3" s="1"/>
+      <c r="N3" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>30</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="G4" s="1"/>
       <c r="H4" s="1" t="s">
         <v>31</v>
       </c>
@@ -638,29 +698,35 @@
       <c r="J4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
+      <c r="K4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="1"/>
+        <v>17</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="F5" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>37</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="G5" s="1"/>
       <c r="H5" s="1" t="s">
         <v>38</v>
       </c>
@@ -670,9 +736,133 @@
       <c r="J5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="K5" s="1"/>
+      <c r="K5" s="1" t="s">
+        <v>41</v>
+      </c>
       <c r="L5" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M6" s="1"/>
+      <c r="N6" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M8" s="1"/>
+      <c r="N8" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update account test cases and user.json
</commit_message>
<xml_diff>
--- a/data/test_cases/account_test_cases.xlsx
+++ b/data/test_cases/account_test_cases.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="57">
   <si>
     <t>case_no</t>
   </si>
@@ -103,9 +103,6 @@
     <t>/api/accounts/{admin_account_id}</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Account03</t>
   </si>
   <si>
@@ -127,6 +124,9 @@
     <t>Account04</t>
   </si>
   <si>
+    <t>Skip</t>
+  </si>
+  <si>
     <t>major</t>
   </si>
   <si>
@@ -169,6 +169,9 @@
     <t>Account07</t>
   </si>
   <si>
+    <t>Failed</t>
+  </si>
+  <si>
     <t>negative</t>
   </si>
   <si>
@@ -179,6 +182,9 @@
   </si>
   <si>
     <t>{"status_code":401}</t>
+  </si>
+  <si>
+    <t>2026-01-08: [FAILED] Status code is not equal. Expected: 401, Actual: 200. Detail message:</t>
   </si>
 </sst>
 </file>
@@ -215,12 +221,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -531,20 +534,20 @@
   <dimension ref="A1:N8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="10.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="3" width="7.433571428571429" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="3" width="8.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="3" width="13.576428571428572" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="8" max="8" style="3" width="49.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="3" width="10.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="3" width="29.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="3" width="340.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="3" width="51.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="3" width="47.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="2" width="10.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="2" width="7.433571428571429" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="2" width="8.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="2" width="13.576428571428572" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="8" max="8" style="2" width="49.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="2" width="10.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="2" width="29.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="2" width="340.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="2" width="51.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="2" width="47.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -665,13 +668,11 @@
         <v>24</v>
       </c>
       <c r="M3" s="1"/>
-      <c r="N3" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="N3" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>15</v>
@@ -690,29 +691,29 @@
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>37</v>
@@ -766,9 +767,7 @@
       <c r="F6" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="G6" s="1"/>
       <c r="H6" s="1" t="s">
         <v>46</v>
       </c>
@@ -778,16 +777,12 @@
       <c r="J6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="K6" s="1"/>
       <c r="L6" s="1" t="s">
         <v>24</v>
       </c>
       <c r="M6" s="1"/>
-      <c r="N6" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="N6" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1" t="s">
@@ -830,13 +825,13 @@
         <v>50</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>15</v>
+        <v>51</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>18</v>
@@ -846,23 +841,23 @@
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="J8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="J8" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="K8" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M8" s="1"/>
-      <c r="N8" s="2" t="s">
-        <v>29</v>
+      <c r="N8" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
setup and run on local computer
</commit_message>
<xml_diff>
--- a/data/test_cases/account_test_cases.xlsx
+++ b/data/test_cases/account_test_cases.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="56">
   <si>
     <t>case_no</t>
   </si>
@@ -61,7 +61,7 @@
     <t>Account01</t>
   </si>
   <si>
-    <t>Done</t>
+    <t>Skip</t>
   </si>
   <si>
     <t>critical</t>
@@ -122,9 +122,6 @@
   </si>
   <si>
     <t>Account04</t>
-  </si>
-  <si>
-    <t>Skip</t>
   </si>
   <si>
     <t>major</t>
@@ -713,10 +710,10 @@
         <v>35</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>37</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>17</v>
@@ -729,34 +726,34 @@
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="K5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="L5" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="M5" s="1"/>
       <c r="N5" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>17</v>
@@ -765,11 +762,11 @@
         <v>18</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>22</v>
@@ -786,13 +783,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>17</v>
@@ -801,11 +798,11 @@
         <v>18</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>22</v>
@@ -822,26 +819,26 @@
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>52</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>18</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>31</v>
@@ -850,14 +847,14 @@
         <v>32</v>
       </c>
       <c r="K8" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="L8" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="M8" s="1"/>
       <c r="N8" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update code and test case
</commit_message>
<xml_diff>
--- a/data/test_cases/account_test_cases.xlsx
+++ b/data/test_cases/account_test_cases.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="54">
   <si>
     <t>case_no</t>
   </si>
@@ -61,69 +61,72 @@
     <t>Account01</t>
   </si>
   <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>critical</t>
+  </si>
+  <si>
+    <t>positive</t>
+  </si>
+  <si>
+    <t>Nhat</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>GetAllRoles</t>
+  </si>
+  <si>
+    <t>Get all accounts.</t>
+  </si>
+  <si>
+    <t>GET</t>
+  </si>
+  <si>
+    <t>/api/accounts</t>
+  </si>
+  <si>
+    <t>{"_id":"{admin_account_id}","status_code":200}</t>
+  </si>
+  <si>
+    <t>Account02</t>
+  </si>
+  <si>
+    <t>GetRoleById</t>
+  </si>
+  <si>
+    <t>Get account by id.</t>
+  </si>
+  <si>
+    <t>/api/accounts/{admin_account_id}</t>
+  </si>
+  <si>
+    <t>Account03</t>
+  </si>
+  <si>
+    <t>Create new account with role admin.</t>
+  </si>
+  <si>
+    <t>POST</t>
+  </si>
+  <si>
+    <t>/api/auth/register</t>
+  </si>
+  <si>
+    <t>{"role_name": "{student_role_name}", "full_name": "API csv - student account 01", "date_of_birth": "2022-01-25", "gender": "nam", "address": "API csv - student account 01 - address", "email": "api_csv_student_account_01@gmail.com", "phone_number": "1234567890", "password": "123456789", "confirmPassword": "123456789"}</t>
+  </si>
+  <si>
+    <t>{"status_code":200}</t>
+  </si>
+  <si>
+    <t>Account04</t>
+  </si>
+  <si>
     <t>Skip</t>
   </si>
   <si>
-    <t>critical</t>
-  </si>
-  <si>
-    <t>positive</t>
-  </si>
-  <si>
-    <t>Nhat</t>
-  </si>
-  <si>
-    <t>admin</t>
-  </si>
-  <si>
-    <t>GetAllRoles</t>
-  </si>
-  <si>
-    <t>Get all accounts.</t>
-  </si>
-  <si>
-    <t>GET</t>
-  </si>
-  <si>
-    <t>/api/accounts</t>
-  </si>
-  <si>
-    <t>{"_id":"{admin_account_id}","status_code":200}</t>
-  </si>
-  <si>
-    <t>Account02</t>
-  </si>
-  <si>
-    <t>GetRoleById</t>
-  </si>
-  <si>
-    <t>Get account by id.</t>
-  </si>
-  <si>
-    <t>/api/accounts/{admin_account_id}</t>
-  </si>
-  <si>
-    <t>Account03</t>
-  </si>
-  <si>
-    <t>Create new account with role admin.</t>
-  </si>
-  <si>
-    <t>POST</t>
-  </si>
-  <si>
-    <t>/api/auth/register</t>
-  </si>
-  <si>
-    <t>{"role_name": "{student_role_name}", "full_name": "API csv - student account 01", "date_of_birth": "2022-01-25", "gender": "nam", "address": "API csv - student account 01 - address", "email": "api_csv_student_account_01@gmail.com", "phone_number": "1234567890", "password": "123456789", "confirmPassword": "123456789"}</t>
-  </si>
-  <si>
-    <t>{"status_code":200}</t>
-  </si>
-  <si>
-    <t>Account04</t>
-  </si>
-  <si>
     <t>major</t>
   </si>
   <si>
@@ -166,22 +169,13 @@
     <t>Account07</t>
   </si>
   <si>
-    <t>Failed</t>
-  </si>
-  <si>
-    <t>negative</t>
-  </si>
-  <si>
     <t>Create new account with role teacher.</t>
   </si>
   <si>
     <t>{"role_name": "{student_role_name}", "full_name": "API csv - student account 02", "date_of_birth": "2022-01-25", "gender": "nam", "address": "API csv - student account 02 - address", "email": "api_csv_student_account_02@gmail.com", "phone_number": "1234567890", "password": "123456789", "confirmPassword": "123456789"}</t>
   </si>
   <si>
-    <t>{"status_code":401}</t>
-  </si>
-  <si>
-    <t>2026-01-08: [FAILED] Status code is not equal. Expected: 401, Actual: 200. Detail message:</t>
+    <t/>
   </si>
 </sst>
 </file>
@@ -218,9 +212,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -531,20 +528,20 @@
   <dimension ref="A1:N8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="2" width="10.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="2" width="7.433571428571429" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="2" width="8.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="2" width="13.576428571428572" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="8" max="8" style="2" width="49.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="2" width="10.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="2" width="29.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="2" width="340.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="2" width="51.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="2" width="47.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="3" width="10.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="3" width="7.433571428571429" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="3" width="8.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="3" width="13.576428571428572" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="8" max="8" style="3" width="49.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="3" width="10.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="3" width="29.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="3" width="340.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="3" width="51.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="3" width="47.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -710,10 +707,10 @@
         <v>35</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>17</v>
@@ -726,34 +723,34 @@
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="M5" s="1"/>
       <c r="N5" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>17</v>
@@ -762,11 +759,11 @@
         <v>18</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>22</v>
@@ -783,13 +780,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>17</v>
@@ -798,11 +795,11 @@
         <v>18</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>22</v>
@@ -819,26 +816,26 @@
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>18</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>31</v>
@@ -847,14 +844,14 @@
         <v>32</v>
       </c>
       <c r="K8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M8" s="1"/>
+      <c r="N8" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1" t="s">
-        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>